<commit_message>
Features/boss effect qa (#102)
* Outline을 이용한 차징시 빨간 외곽선 처리

ChargedCombo 부분 숨고르기 애니메이션 짧게 수정

* 보스용 Asset 데이터 추가

* 보스 피격처리 관련 작업 진행중

* Hit VFX 처리

* Asset 추가 무기

* 보스 트레일 작업

* 보스 접근 최소 거리 지정 및 차징시 이펙트 Loop 처리

* 광역공격 이펙트 처리

* 플레이어 사망시 보스 Idle 상태 유지 보스 데미지 조정

* PlayRate 작업 및 몽타주 수정 작업 일부
</commit_message>
<xml_diff>
--- a/BADesign/Excel/BossMonster.xlsx
+++ b/BADesign/Excel/BossMonster.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="Polaris Office Sheet" lastEdited="4" lowestEdited="4" rupBuild="10.105.293.56114"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="30" windowWidth="25755" windowHeight="11595" tabRatio="460" activeTab="0"/>
+    <workbookView xWindow="360" yWindow="30" windowWidth="25755" windowHeight="11595" tabRatio="450" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="1StageBossAttack" sheetId="1" r:id="rId1"/>
@@ -1319,10 +1319,10 @@
         <v>24</v>
       </c>
       <c r="P3" s="3">
-        <v>150</v>
+        <v>300</v>
       </c>
       <c r="Q3" s="3">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="R3" s="3">
         <v>0</v>
@@ -1388,10 +1388,10 @@
         <v>26</v>
       </c>
       <c r="P4" s="3">
-        <v>200</v>
+        <v>330</v>
       </c>
       <c r="Q4" s="3">
-        <v>20</v>
+        <v>34</v>
       </c>
       <c r="R4" s="3">
         <v>0</v>
@@ -1526,10 +1526,10 @@
         <v>30</v>
       </c>
       <c r="P6" s="3">
-        <v>220</v>
+        <v>320</v>
       </c>
       <c r="Q6" s="3">
-        <v>40</v>
+        <v>67</v>
       </c>
       <c r="R6" s="3"/>
       <c r="S6" s="3">
@@ -1593,10 +1593,10 @@
         <v>32</v>
       </c>
       <c r="P7" s="3">
-        <v>300</v>
+        <v>9999</v>
       </c>
       <c r="Q7" s="3">
-        <v>160</v>
+        <v>0</v>
       </c>
       <c r="R7" s="3">
         <v>108</v>
@@ -1665,7 +1665,7 @@
         <v>250</v>
       </c>
       <c r="Q8" s="3">
-        <v>80</v>
+        <v>134</v>
       </c>
       <c r="R8" s="3">
         <v>0</v>
@@ -1731,10 +1731,10 @@
         <v>36</v>
       </c>
       <c r="P9" s="3">
-        <v>150</v>
+        <v>300</v>
       </c>
       <c r="Q9" s="3">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="R9" s="3">
         <v>0</v>
@@ -1800,10 +1800,10 @@
         <v>38</v>
       </c>
       <c r="P10" s="3">
-        <v>150</v>
+        <v>300</v>
       </c>
       <c r="Q10" s="3">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="R10" s="3">
         <v>0</v>
@@ -1872,7 +1872,7 @@
         <v>9999</v>
       </c>
       <c r="Q11" s="3">
-        <v>350</v>
+        <v>150</v>
       </c>
       <c r="R11" s="3">
         <v>0</v>

</xml_diff>